<commit_message>
Add Neil Optimistic scenario (G2 RNm 10km) to map and model
</commit_message>
<xml_diff>
--- a/WeLink_AZ_BEAD_CAPEX_OPEX_Model.xlsx
+++ b/WeLink_AZ_BEAD_CAPEX_OPEX_Model.xlsx
@@ -12,10 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corrected Design" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Optimized Design" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neil Hybrid" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues Found" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Neil Optimistic" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues Found" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="166" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="167" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -145,6 +146,21 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00CC0000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -196,7 +212,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -365,6 +381,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1787,6 +1808,317 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <tabColor rgb="FFFF0000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="6" customWidth="1" style="27" min="1" max="1"/>
+    <col width="40" customWidth="1" style="27" min="2" max="2"/>
+    <col width="50" customWidth="1" style="27" min="3" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.25" customHeight="1" s="28">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>Audit Issues Found</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="28">
+      <c r="A3" s="60" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="C3" s="60" t="inlineStr">
+        <is>
+          <t>Why It Matters</t>
+        </is>
+      </c>
+      <c r="D3" s="60" t="inlineStr">
+        <is>
+          <t>Fix Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1" s="28">
+      <c r="A4" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="61" t="inlineStr">
+        <is>
+          <t>Comparison sheet references broken</t>
+        </is>
+      </c>
+      <c r="C4" s="61" t="inlineStr">
+        <is>
+          <t>Row insertions for Ketsen data shifted cell refs. Corrected BSLs showed 13 instead of 11,346. Optimized CAPEX showed $600K (coloc only). All downstream Comparison values wrong.</t>
+        </is>
+      </c>
+      <c r="D4" s="61" t="inlineStr">
+        <is>
+          <t>Rebuilt Comparison with correct cross-sheet refs to new row layout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1" s="28">
+      <c r="A5" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>Sector equipment CAPEX never used</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>Assumptions had $50K/sector for Tarana G2 BN but no scenario formula used it. Infrastructure CAPEX was either hardcoded or only counted tower build costs. Understated CAPEX by $2-3M.</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Replaced with architecture-driven CAPEX: G2 BN at $21K/sector + $11,634/P2P BH sector + per-site accessories, all formula-linked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1" s="28">
+      <c r="A6" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="61" t="inlineStr">
+        <is>
+          <t>Corrected Design Infra CAPEX hardcoded</t>
+        </is>
+      </c>
+      <c r="C6" s="61" t="inlineStr">
+        <is>
+          <t>$5,076,000 hardcoded with no formula decomposition. Cannot audit, cannot sensitivity-test, cannot tie to architecture.</t>
+        </is>
+      </c>
+      <c r="D6" s="61" t="inlineStr">
+        <is>
+          <t>Replaced with formula: sectors*BN + P2P*BH + sites*accessories + gateways + tower build + make-ready + contingency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1" s="28">
+      <c r="A7" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>Current Design Infra CAPEX hardcoded</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>$3,260,000 with no formula basis. Board/lender cannot verify.</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Replaced with formula-driven CAPEX built from sector count, per-site accessories, make-ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1" s="28">
+      <c r="A8" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="61" t="inlineStr">
+        <is>
+          <t>OPEX was 10% of revenue</t>
+        </is>
+      </c>
+      <c r="C8" s="61" t="inlineStr">
+        <is>
+          <t>Completely unrealistic. At 5% take rate in Y1, total OPEX would be ~$40K while tower leases alone are $720K+. Understated early-year OPEX by 10-20x, overstated EBITDA.</t>
+        </is>
+      </c>
+      <c r="D8" s="61" t="inlineStr">
+        <is>
+          <t>Replaced with 10-line itemized OPEX: leases, power, NOC, transport, field maintenance, customer support, SMS, SAS, insurance, spares. Each linked to Assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1" s="28">
+      <c r="A9" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>Tower leases wrong for Corrected Design</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>All 101 sites used New Tower Lease ($24K/yr). Should differentiate coloc vs new build. Overstated Corrected lease expense.</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>Corrected: all new build at $6K ground lease. Optimized: split 24 coloc at $18K + 77 new at $6K.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1" s="28">
+      <c r="A10" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="61" t="inlineStr">
+        <is>
+          <t>No BEAD draw timing or retainage</t>
+        </is>
+      </c>
+      <c r="C10" s="61" t="inlineStr">
+        <is>
+          <t>Model assumed full P4 in Y1, full P5 in Y2. Real BEAD has milestone-based draws and 10% retainage until closeout. Overstated early cash position.</t>
+        </is>
+      </c>
+      <c r="D10" s="61" t="inlineStr">
+        <is>
+          <t>Added retainage assumption (10%), draw timing schedule (40/30/20/10%), retainage release in Y4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1" s="28">
+      <c r="A11" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>No contingency in CAPEX</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>Zero contingency on a 101-site new build across Maricopa County. No buffer for permitting, weather, supply chain. Not defensible for board or state review.</t>
+        </is>
+      </c>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>Added 10% contingency on pre-contingency infrastructure CAPEX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1" s="28">
+      <c r="A12" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="61" t="inlineStr">
+        <is>
+          <t>CPE cost not split by technology</t>
+        </is>
+      </c>
+      <c r="C12" s="61" t="inlineStr">
+        <is>
+          <t>Uniform $705/sub CPE for all BSLs. Ketsen mesh CPE is likely cheaper than Tarana G2 RN.</t>
+        </is>
+      </c>
+      <c r="D12" s="61" t="inlineStr">
+        <is>
+          <t>Split CPE: Tarana at $705 (RNv $455 + BW $100 + Install $150), Ketsen at $350 ($250 + $100).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1" s="28">
+      <c r="A13" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>No technology-segmented take rates</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>One take rate for all BSLs regardless of architecture. Dense Ketsen areas may have different adoption curves.</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>Added separate Tarana and Ketsen take rate columns in Assumptions. Ketsen rates slightly lower to reflect density/competition dynamics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1" s="28">
+      <c r="A14" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="61" t="inlineStr">
+        <is>
+          <t>Map economics fully hardcoded</t>
+        </is>
+      </c>
+      <c r="C14" s="61" t="inlineStr">
+        <is>
+          <t>All KPI badges, economics panels, and CAPEX bar charts are hardcoded HTML strings. Any model change requires manual map edit.</t>
+        </is>
+      </c>
+      <c r="D14" s="61" t="inlineStr">
+        <is>
+          <t>Documented. Map should be updated to read from a JSON export or the model directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1" s="28">
+      <c r="A15" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>Sector equipment assumption mislabeled</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>Assumptions showed "Sector Equipment (Tarana G2 BN + BH)" at $50K. Actual G2 BN is $21K. $50K was never used anyway.</t>
+        </is>
+      </c>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>Replaced with actual Tarana pricing: G2 BN $21K/sector, P2P BH $11,634/sector, per-site accessories $1,446.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1" s="28">
+      <c r="A16" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="61" t="inlineStr">
+        <is>
+          <t>No OPEX escalator</t>
+        </is>
+      </c>
+      <c r="C16" s="61" t="inlineStr">
+        <is>
+          <t>Fixed costs assumed flat for 5 years. Tower leases, power, labor all inflate.</t>
+        </is>
+      </c>
+      <c r="D16" s="61" t="inlineStr">
+        <is>
+          <t>Added 3% annual escalator on fixed OPEX items.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -5468,6 +5800,573 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" style="28" min="1" max="1"/>
+    <col width="18" customWidth="1" style="28" min="2" max="2"/>
+    <col width="14" customWidth="1" style="28" min="3" max="3"/>
+    <col width="14" customWidth="1" style="28" min="4" max="4"/>
+    <col width="14" customWidth="1" style="28" min="5" max="5"/>
+    <col width="18" customWidth="1" style="28" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="62" t="inlineStr">
+        <is>
+          <t>Neil Optimistic Design Scenario (G2 RNm 10km)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="63" t="inlineStr">
+        <is>
+          <t>WARNING: Requires field validation of 10km RNm link budgets from elevation sites. Uses CBRS + 6 GHz (160 MHz) spec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="64" t="inlineStr">
+        <is>
+          <t>SITE CONFIGURATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Neil Anchor Sites (active)</t>
+        </is>
+      </c>
+      <c r="B5" s="65" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ELNK Building Colocations</t>
+        </is>
+      </c>
+      <c r="B6" s="65" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ASR Tower Colocations</t>
+        </is>
+      </c>
+      <c r="B7" s="65" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Neil New Builds (elevation)</t>
+        </is>
+      </c>
+      <c r="B8" s="65" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Infill Sites (coverage gaps)</t>
+        </is>
+      </c>
+      <c r="B9" s="65" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sites Removed (0 BSLs)</t>
+        </is>
+      </c>
+      <c r="B10" s="65" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Total Active Sites</t>
+        </is>
+      </c>
+      <c r="B11" s="65" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Total Colocation</t>
+        </is>
+      </c>
+      <c r="B12" s="65" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Total New Build</t>
+        </is>
+      </c>
+      <c r="B13" s="65" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="64" t="inlineStr">
+        <is>
+          <t>NETWORK ARCHITECTURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>G2 RNm Access Sectors</t>
+        </is>
+      </c>
+      <c r="B16" s="65" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P2P Backhaul Links</t>
+        </is>
+      </c>
+      <c r="B17" s="65" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ketsen Gateways</t>
+        </is>
+      </c>
+      <c r="B18" s="65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BSLs Covered</t>
+        </is>
+      </c>
+      <c r="B19" s="65" t="n">
+        <v>11346</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Avg Sectors/Site</t>
+        </is>
+      </c>
+      <c r="B20" s="65" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Range Assumption</t>
+        </is>
+      </c>
+      <c r="B21" s="65" t="inlineStr">
+        <is>
+          <t>10km (G2 BN-RNm, CBRS + 6 GHz, elevation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="64" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>G2 RNm BNs (98 x $21K)</t>
+        </is>
+      </c>
+      <c r="B24" s="66" t="n">
+        <v>2058000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>P2P BH (35 x $11.6K)</t>
+        </is>
+      </c>
+      <c r="B25" s="66" t="n">
+        <v>407190</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Accessories (35 x $1.4K)</t>
+        </is>
+      </c>
+      <c r="B26" s="66" t="n">
+        <v>50610</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ketsen GW (0)</t>
+        </is>
+      </c>
+      <c r="B27" s="66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Equipment Subtotal</t>
+        </is>
+      </c>
+      <c r="B28" s="66" t="n">
+        <v>2515800</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Coloc Setup (19 x $25K)</t>
+        </is>
+      </c>
+      <c r="B30" s="66" t="n">
+        <v>475000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>New Towers (16 x $50K)</t>
+        </is>
+      </c>
+      <c r="B31" s="66" t="n">
+        <v>800000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Make-Ready (19 x $10K)</t>
+        </is>
+      </c>
+      <c r="B32" s="66" t="n">
+        <v>190000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Infrastructure Subtotal</t>
+        </is>
+      </c>
+      <c r="B33" s="66" t="n">
+        <v>1465000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B35" s="66" t="n">
+        <v>3980800</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Contingency (10%)</t>
+        </is>
+      </c>
+      <c r="B36" s="66" t="n">
+        <v>398080</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>TOTAL CAPEX</t>
+        </is>
+      </c>
+      <c r="B37" s="66" t="n">
+        <v>4378880</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="64" t="inlineStr">
+        <is>
+          <t>ANNUAL LEASE OPEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Coloc Leases (19 x $18K)</t>
+        </is>
+      </c>
+      <c r="B40" s="66" t="n">
+        <v>342000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Ground Leases (16 x $6K)</t>
+        </is>
+      </c>
+      <c r="B41" s="66" t="n">
+        <v>96000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Total Lease OPEX</t>
+        </is>
+      </c>
+      <c r="B42" s="66" t="n">
+        <v>438000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="64" t="inlineStr">
+        <is>
+          <t>COMPARISON</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="65" t="inlineStr"/>
+      <c r="B45" s="65" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C45" s="65" t="inlineStr">
+        <is>
+          <t>Corrected</t>
+        </is>
+      </c>
+      <c r="D45" s="65" t="inlineStr">
+        <is>
+          <t>Optimized</t>
+        </is>
+      </c>
+      <c r="E45" s="65" t="inlineStr">
+        <is>
+          <t>Neil Hybrid</t>
+        </is>
+      </c>
+      <c r="F45" s="65" t="inlineStr">
+        <is>
+          <t>Neil Optimistic</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sites</t>
+        </is>
+      </c>
+      <c r="B46" s="65" t="n">
+        <v>6</v>
+      </c>
+      <c r="C46" s="65" t="n">
+        <v>101</v>
+      </c>
+      <c r="D46" s="65" t="n">
+        <v>101</v>
+      </c>
+      <c r="E46" s="65" t="n">
+        <v>100</v>
+      </c>
+      <c r="F46" s="65" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Sectors</t>
+        </is>
+      </c>
+      <c r="B47" s="65" t="n">
+        <v>80</v>
+      </c>
+      <c r="C47" s="65" t="n">
+        <v>115</v>
+      </c>
+      <c r="D47" s="65" t="n">
+        <v>115</v>
+      </c>
+      <c r="E47" s="65" t="n">
+        <v>181</v>
+      </c>
+      <c r="F47" s="65" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BSLs</t>
+        </is>
+      </c>
+      <c r="B48" s="65" t="n">
+        <v>9584</v>
+      </c>
+      <c r="C48" s="65" t="n">
+        <v>11346</v>
+      </c>
+      <c r="D48" s="65" t="n">
+        <v>11346</v>
+      </c>
+      <c r="E48" s="65" t="n">
+        <v>11346</v>
+      </c>
+      <c r="F48" s="65" t="n">
+        <v>11346</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Infra CAPEX</t>
+        </is>
+      </c>
+      <c r="B49" s="66" t="n">
+        <v>2378024</v>
+      </c>
+      <c r="C49" s="66" t="n">
+        <v>9377817</v>
+      </c>
+      <c r="D49" s="66" t="n">
+        <v>8717817</v>
+      </c>
+      <c r="E49" s="66" t="n">
+        <v>10914200</v>
+      </c>
+      <c r="F49" s="66" t="n">
+        <v>4378880</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Lease OPEX/yr</t>
+        </is>
+      </c>
+      <c r="B50" s="66" t="n">
+        <v>720000</v>
+      </c>
+      <c r="C50" s="66" t="n">
+        <v>606000</v>
+      </c>
+      <c r="D50" s="66" t="n">
+        <v>894000</v>
+      </c>
+      <c r="E50" s="66" t="n">
+        <v>780000</v>
+      </c>
+      <c r="F50" s="66" t="n">
+        <v>438000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="64" t="inlineStr">
+        <is>
+          <t>KEY FINDINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>At 10km RNm range, only 7 infill sites needed (vs 76 at 5km) for 100% BSL coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Total CAPEX $4.38M, roughly $5M below Corrected design</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Only 98 sectors required vs 181 (Neil Hybrid) and 115 (Corrected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Lease OPEX $438K/yr, lowest of any full-coverage scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>19 coloc sites leverage existing ELNK + ASR infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CRITICAL: 10km range from elevation requires field validation with G2 BN-RNm hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Risk: If field tests show &lt;8km reliable range, additional infill sites will be needed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="FF4472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5845,7 +6744,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="FFFF6600"/>
@@ -6267,7 +7166,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="FF7030A0"/>
@@ -6609,315 +7508,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <tabColor rgb="FFFF0000"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="6" customWidth="1" style="27" min="1" max="1"/>
-    <col width="40" customWidth="1" style="27" min="2" max="2"/>
-    <col width="50" customWidth="1" style="27" min="3" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="17.25" customHeight="1" s="28">
-      <c r="A1" s="29" t="inlineStr">
-        <is>
-          <t>Audit Issues Found</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="28">
-      <c r="A3" s="60" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B3" s="60" t="inlineStr">
-        <is>
-          <t>Issue</t>
-        </is>
-      </c>
-      <c r="C3" s="60" t="inlineStr">
-        <is>
-          <t>Why It Matters</t>
-        </is>
-      </c>
-      <c r="D3" s="60" t="inlineStr">
-        <is>
-          <t>Fix Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="45" customHeight="1" s="28">
-      <c r="A4" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="61" t="inlineStr">
-        <is>
-          <t>Comparison sheet references broken</t>
-        </is>
-      </c>
-      <c r="C4" s="61" t="inlineStr">
-        <is>
-          <t>Row insertions for Ketsen data shifted cell refs. Corrected BSLs showed 13 instead of 11,346. Optimized CAPEX showed $600K (coloc only). All downstream Comparison values wrong.</t>
-        </is>
-      </c>
-      <c r="D4" s="61" t="inlineStr">
-        <is>
-          <t>Rebuilt Comparison with correct cross-sheet refs to new row layout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="45" customHeight="1" s="28">
-      <c r="A5" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="61" t="inlineStr">
-        <is>
-          <t>Sector equipment CAPEX never used</t>
-        </is>
-      </c>
-      <c r="C5" s="61" t="inlineStr">
-        <is>
-          <t>Assumptions had $50K/sector for Tarana G2 BN but no scenario formula used it. Infrastructure CAPEX was either hardcoded or only counted tower build costs. Understated CAPEX by $2-3M.</t>
-        </is>
-      </c>
-      <c r="D5" s="61" t="inlineStr">
-        <is>
-          <t>Replaced with architecture-driven CAPEX: G2 BN at $21K/sector + $11,634/P2P BH sector + per-site accessories, all formula-linked.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1" s="28">
-      <c r="A6" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="61" t="inlineStr">
-        <is>
-          <t>Corrected Design Infra CAPEX hardcoded</t>
-        </is>
-      </c>
-      <c r="C6" s="61" t="inlineStr">
-        <is>
-          <t>$5,076,000 hardcoded with no formula decomposition. Cannot audit, cannot sensitivity-test, cannot tie to architecture.</t>
-        </is>
-      </c>
-      <c r="D6" s="61" t="inlineStr">
-        <is>
-          <t>Replaced with formula: sectors*BN + P2P*BH + sites*accessories + gateways + tower build + make-ready + contingency.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1" s="28">
-      <c r="A7" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="61" t="inlineStr">
-        <is>
-          <t>Current Design Infra CAPEX hardcoded</t>
-        </is>
-      </c>
-      <c r="C7" s="61" t="inlineStr">
-        <is>
-          <t>$3,260,000 with no formula basis. Board/lender cannot verify.</t>
-        </is>
-      </c>
-      <c r="D7" s="61" t="inlineStr">
-        <is>
-          <t>Replaced with formula-driven CAPEX built from sector count, per-site accessories, make-ready.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1" s="28">
-      <c r="A8" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="61" t="inlineStr">
-        <is>
-          <t>OPEX was 10% of revenue</t>
-        </is>
-      </c>
-      <c r="C8" s="61" t="inlineStr">
-        <is>
-          <t>Completely unrealistic. At 5% take rate in Y1, total OPEX would be ~$40K while tower leases alone are $720K+. Understated early-year OPEX by 10-20x, overstated EBITDA.</t>
-        </is>
-      </c>
-      <c r="D8" s="61" t="inlineStr">
-        <is>
-          <t>Replaced with 10-line itemized OPEX: leases, power, NOC, transport, field maintenance, customer support, SMS, SAS, insurance, spares. Each linked to Assumptions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1" s="28">
-      <c r="A9" s="32" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="61" t="inlineStr">
-        <is>
-          <t>Tower leases wrong for Corrected Design</t>
-        </is>
-      </c>
-      <c r="C9" s="61" t="inlineStr">
-        <is>
-          <t>All 101 sites used New Tower Lease ($24K/yr). Should differentiate coloc vs new build. Overstated Corrected lease expense.</t>
-        </is>
-      </c>
-      <c r="D9" s="61" t="inlineStr">
-        <is>
-          <t>Corrected: all new build at $6K ground lease. Optimized: split 24 coloc at $18K + 77 new at $6K.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1" s="28">
-      <c r="A10" s="32" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="61" t="inlineStr">
-        <is>
-          <t>No BEAD draw timing or retainage</t>
-        </is>
-      </c>
-      <c r="C10" s="61" t="inlineStr">
-        <is>
-          <t>Model assumed full P4 in Y1, full P5 in Y2. Real BEAD has milestone-based draws and 10% retainage until closeout. Overstated early cash position.</t>
-        </is>
-      </c>
-      <c r="D10" s="61" t="inlineStr">
-        <is>
-          <t>Added retainage assumption (10%), draw timing schedule (40/30/20/10%), retainage release in Y4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1" s="28">
-      <c r="A11" s="32" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="61" t="inlineStr">
-        <is>
-          <t>No contingency in CAPEX</t>
-        </is>
-      </c>
-      <c r="C11" s="61" t="inlineStr">
-        <is>
-          <t>Zero contingency on a 101-site new build across Maricopa County. No buffer for permitting, weather, supply chain. Not defensible for board or state review.</t>
-        </is>
-      </c>
-      <c r="D11" s="61" t="inlineStr">
-        <is>
-          <t>Added 10% contingency on pre-contingency infrastructure CAPEX.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1" s="28">
-      <c r="A12" s="32" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="61" t="inlineStr">
-        <is>
-          <t>CPE cost not split by technology</t>
-        </is>
-      </c>
-      <c r="C12" s="61" t="inlineStr">
-        <is>
-          <t>Uniform $705/sub CPE for all BSLs. Ketsen mesh CPE is likely cheaper than Tarana G2 RN.</t>
-        </is>
-      </c>
-      <c r="D12" s="61" t="inlineStr">
-        <is>
-          <t>Split CPE: Tarana at $705 (RNv $455 + BW $100 + Install $150), Ketsen at $350 ($250 + $100).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1" s="28">
-      <c r="A13" s="32" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="61" t="inlineStr">
-        <is>
-          <t>No technology-segmented take rates</t>
-        </is>
-      </c>
-      <c r="C13" s="61" t="inlineStr">
-        <is>
-          <t>One take rate for all BSLs regardless of architecture. Dense Ketsen areas may have different adoption curves.</t>
-        </is>
-      </c>
-      <c r="D13" s="61" t="inlineStr">
-        <is>
-          <t>Added separate Tarana and Ketsen take rate columns in Assumptions. Ketsen rates slightly lower to reflect density/competition dynamics.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1" s="28">
-      <c r="A14" s="32" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="61" t="inlineStr">
-        <is>
-          <t>Map economics fully hardcoded</t>
-        </is>
-      </c>
-      <c r="C14" s="61" t="inlineStr">
-        <is>
-          <t>All KPI badges, economics panels, and CAPEX bar charts are hardcoded HTML strings. Any model change requires manual map edit.</t>
-        </is>
-      </c>
-      <c r="D14" s="61" t="inlineStr">
-        <is>
-          <t>Documented. Map should be updated to read from a JSON export or the model directly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="45" customHeight="1" s="28">
-      <c r="A15" s="32" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="61" t="inlineStr">
-        <is>
-          <t>Sector equipment assumption mislabeled</t>
-        </is>
-      </c>
-      <c r="C15" s="61" t="inlineStr">
-        <is>
-          <t>Assumptions showed "Sector Equipment (Tarana G2 BN + BH)" at $50K. Actual G2 BN is $21K. $50K was never used anyway.</t>
-        </is>
-      </c>
-      <c r="D15" s="61" t="inlineStr">
-        <is>
-          <t>Replaced with actual Tarana pricing: G2 BN $21K/sector, P2P BH $11,634/sector, per-site accessories $1,446.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1" s="28">
-      <c r="A16" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="61" t="inlineStr">
-        <is>
-          <t>No OPEX escalator</t>
-        </is>
-      </c>
-      <c r="C16" s="61" t="inlineStr">
-        <is>
-          <t>Fixed costs assumed flat for 5 years. Tower leases, power, labor all inflate.</t>
-        </is>
-      </c>
-      <c r="D16" s="61" t="inlineStr">
-        <is>
-          <t>Added 3% annual escalator on fixed OPEX items.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
 </file>
</xml_diff>